<commit_message>
Fix in some models
</commit_message>
<xml_diff>
--- a/db/portfolio_db.xlsx
+++ b/db/portfolio_db.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Bridge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0C2DAFBA-65B7-41C3-847E-741E9D0D00B9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BC28926-4B0A-43C5-8B60-1BEEC8E0E240}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{5F6615A1-1CC4-4DED-9F3A-C4C5BF29ED5B}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{5F6615A1-1CC4-4DED-9F3A-C4C5BF29ED5B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="67">
   <si>
     <t>Summary</t>
   </si>
@@ -48,15 +48,6 @@
     <t>education[]</t>
   </si>
   <si>
-    <t>Awards</t>
-  </si>
-  <si>
-    <t>miscellaneous[]</t>
-  </si>
-  <si>
-    <t>Miscellaneous</t>
-  </si>
-  <si>
     <t>number</t>
   </si>
   <si>
@@ -90,9 +81,6 @@
     <t>Occupation</t>
   </si>
   <si>
-    <t>occupation</t>
-  </si>
-  <si>
     <t>Employer</t>
   </si>
   <si>
@@ -111,9 +99,6 @@
     <t>EndDate</t>
   </si>
   <si>
-    <t>Links</t>
-  </si>
-  <si>
     <t>string[]</t>
   </si>
   <si>
@@ -177,12 +162,12 @@
     <t>Arthur</t>
   </si>
   <si>
+    <t>boolean</t>
+  </si>
+  <si>
     <t>Linkedin</t>
   </si>
   <si>
-    <t>Locale</t>
-  </si>
-  <si>
     <t>Github</t>
   </si>
   <si>
@@ -228,7 +213,19 @@
     <t>Projects</t>
   </si>
   <si>
-    <t>project</t>
+    <t>ExtraInfo</t>
+  </si>
+  <si>
+    <t>extra_infos[]</t>
+  </si>
+  <si>
+    <t>ExtraInfos</t>
+  </si>
+  <si>
+    <t>project[]</t>
+  </si>
+  <si>
+    <t>Continuous</t>
   </si>
 </sst>
 </file>
@@ -597,30 +594,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26F78B82-7883-4188-9D76-B396F717F7A6}">
-  <dimension ref="A1:S27"/>
+  <dimension ref="A1:T27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -636,118 +637,106 @@
       <c r="M1" s="2"/>
       <c r="N1" s="2"/>
       <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2"/>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="P1" s="5"/>
+      <c r="Q1" s="5"/>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>5</v>
+        <v>64</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>12</v>
-      </c>
       <c r="J2" s="3" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>17</v>
+        <v>48</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>6</v>
+        <v>63</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q3" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -769,237 +758,244 @@
       <c r="Q5" s="2"/>
       <c r="R5" s="2"/>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="K6" s="3" t="s">
         <v>0</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="R6" s="3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>21</v>
+        <v>60</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="K7" s="3" t="s">
         <v>1</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="N7" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="P7" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="Q7" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="R7" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>9</v>
+        <v>62</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
-      <c r="H9" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="I9" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="J9" s="2"/>
-      <c r="L9" s="2" t="s">
+      <c r="K9" s="2"/>
+      <c r="M9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="N9" s="2"/>
+      <c r="P9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q9" s="2"/>
+      <c r="S9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="T9" s="2"/>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="M9" s="2"/>
-      <c r="O9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="P9" s="2"/>
-      <c r="R9" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="S9" s="2"/>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>19</v>
-      </c>
       <c r="C10" s="3" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="G10" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="M10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="N10" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="P10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q10" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="I10" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="M10" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="O10" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P10" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="R10" s="3" t="s">
-        <v>33</v>
-      </c>
       <c r="S10" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="T10" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="H11" s="3" t="s">
-        <v>13</v>
+      <c r="G11" s="3" t="s">
+        <v>45</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="L11" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>7</v>
       </c>
       <c r="M11" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="O11" s="3" t="s">
-        <v>13</v>
+      <c r="N11" s="3" t="s">
+        <v>7</v>
       </c>
       <c r="P11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q11" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="R11" s="3" t="s">
-        <v>13</v>
-      </c>
       <c r="S11" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="T11" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="5"/>
       <c r="F13" s="2" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
@@ -1013,106 +1009,106 @@
       <c r="P13" s="2"/>
       <c r="Q13" s="2"/>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="E14" s="5"/>
       <c r="F14" s="3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="N14" s="3" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="O14" s="3" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="P14" s="3" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="Q14" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E15" s="5"/>
       <c r="F15" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>1</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="N15" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="P15" s="3" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="Q15" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="3:17" x14ac:dyDescent="0.25">
@@ -1127,17 +1123,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="R9:S9"/>
     <mergeCell ref="A13:D13"/>
     <mergeCell ref="F13:Q13"/>
-    <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="O9:P9"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="I9:K9"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="P9:Q9"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="G5:K5"/>
     <mergeCell ref="M5:R5"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="S9:T9"/>
+    <mergeCell ref="A1:O1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>